<commit_message>
Finished to review code
</commit_message>
<xml_diff>
--- a/Project/Results.xlsx
+++ b/Project/Results.xlsx
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://polimi365-my.sharepoint.com/personal/10530006_polimi_it/Documents/Work_cloud/DOTTORATO/Robust Optimization/Project/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="4" documentId="13_ncr:1_{AD4E627F-1870-4F48-A017-7A09D30B8898}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{91D09EDD-7623-40D8-B644-AAC366F5B0D1}"/>
+  <xr:revisionPtr revIDLastSave="7" documentId="13_ncr:1_{AD4E627F-1870-4F48-A017-7A09D30B8898}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8ACFA717-1A58-4D47-8BD1-67F0221A4227}"/>
   <bookViews>
-    <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Foglio1" sheetId="1" r:id="rId1"/>
+    <sheet name="Units" sheetId="1" r:id="rId1"/>
     <sheet name="R-LP" sheetId="2" r:id="rId2"/>
     <sheet name="D-LP" sheetId="3" r:id="rId3"/>
     <sheet name="D-LP_real" sheetId="4" r:id="rId4"/>
@@ -129,9 +129,6 @@
     <t>Ct/tonIN</t>
   </si>
   <si>
-    <t>VaR</t>
-  </si>
-  <si>
     <t>VS</t>
   </si>
   <si>
@@ -154,6 +151,9 @@
   </si>
   <si>
     <t>TVFA</t>
+  </si>
+  <si>
+    <t>Prob</t>
   </si>
 </sst>
 </file>
@@ -579,21 +579,21 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:C19"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="17.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.85546875" customWidth="1"/>
+    <col min="1" max="1" width="17.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1"/>
       <c r="B1" s="2"/>
       <c r="C1" s="2" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" s="10" t="s">
         <v>1</v>
       </c>
@@ -602,7 +602,7 @@
       </c>
       <c r="C2" s="3"/>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" s="11" t="s">
         <v>3</v>
       </c>
@@ -611,7 +611,7 @@
       </c>
       <c r="C3" s="6"/>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" s="11" t="s">
         <v>5</v>
       </c>
@@ -620,7 +620,7 @@
       </c>
       <c r="C4" s="6"/>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" s="11" t="s">
         <v>6</v>
       </c>
@@ -629,7 +629,7 @@
       </c>
       <c r="C5" s="6"/>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" s="11" t="s">
         <v>7</v>
       </c>
@@ -638,7 +638,7 @@
       </c>
       <c r="C6" s="6"/>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" s="11" t="s">
         <v>9</v>
       </c>
@@ -647,7 +647,7 @@
       </c>
       <c r="C7" s="6"/>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" s="11" t="s">
         <v>10</v>
       </c>
@@ -656,7 +656,7 @@
       </c>
       <c r="C8" s="6"/>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" s="11" t="s">
         <v>11</v>
       </c>
@@ -665,7 +665,7 @@
       </c>
       <c r="C9" s="6"/>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" s="5" t="s">
         <v>12</v>
       </c>
@@ -674,7 +674,7 @@
       </c>
       <c r="C10" s="7"/>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" s="5" t="s">
         <v>14</v>
       </c>
@@ -683,7 +683,7 @@
       </c>
       <c r="C11" s="7"/>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" s="5" t="s">
         <v>15</v>
       </c>
@@ -692,7 +692,7 @@
       </c>
       <c r="C12" s="7"/>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" s="5" t="s">
         <v>16</v>
       </c>
@@ -701,7 +701,7 @@
       </c>
       <c r="C13" s="7"/>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" s="5" t="s">
         <v>17</v>
       </c>
@@ -710,7 +710,7 @@
       </c>
       <c r="C14" s="7"/>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15" s="5" t="s">
         <v>18</v>
       </c>
@@ -719,7 +719,7 @@
       </c>
       <c r="C15" s="7"/>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16" s="5" t="s">
         <v>19</v>
       </c>
@@ -728,7 +728,7 @@
       </c>
       <c r="C16" s="7"/>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" s="5" t="s">
         <v>20</v>
       </c>
@@ -737,7 +737,7 @@
       </c>
       <c r="C17" s="7"/>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" s="5" t="s">
         <v>21</v>
       </c>
@@ -746,7 +746,7 @@
       </c>
       <c r="C18" s="7"/>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" s="8" t="s">
         <v>22</v>
       </c>
@@ -763,17 +763,17 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:T20"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="19.140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="9" width="10.85546875" bestFit="1" customWidth="1"/>
-    <col min="10" max="17" width="11.85546875" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="10.85546875" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="11.85546875" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="9" width="10.88671875" bestFit="1" customWidth="1"/>
+    <col min="10" max="17" width="11.88671875" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="10.88671875" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="11.88671875" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="10.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -835,7 +835,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="2" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A2" s="11" t="s">
         <v>3</v>
       </c>
@@ -897,7 +897,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A3" s="11" t="s">
         <v>5</v>
       </c>
@@ -959,7 +959,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A4" s="11" t="s">
         <v>6</v>
       </c>
@@ -1021,7 +1021,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="5" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A5" s="11" t="s">
         <v>7</v>
       </c>
@@ -1083,7 +1083,7 @@
         <v>9978.1525846277873</v>
       </c>
     </row>
-    <row r="6" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A6" s="11" t="s">
         <v>9</v>
       </c>
@@ -1145,7 +1145,7 @@
         <v>4959.6784704293632</v>
       </c>
     </row>
-    <row r="7" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A7" s="11" t="s">
         <v>10</v>
       </c>
@@ -1207,7 +1207,7 @@
         <v>894.4298384874013</v>
       </c>
     </row>
-    <row r="8" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A8" s="11" t="s">
         <v>11</v>
       </c>
@@ -1269,7 +1269,7 @@
         <v>4124.0442757110231</v>
       </c>
     </row>
-    <row r="9" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A9" s="5" t="s">
         <v>12</v>
       </c>
@@ -1331,7 +1331,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="10" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A10" s="5" t="s">
         <v>14</v>
       </c>
@@ -1393,7 +1393,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A11" s="5" t="s">
         <v>15</v>
       </c>
@@ -1455,7 +1455,7 @@
         <v>1.78</v>
       </c>
     </row>
-    <row r="12" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A12" s="5" t="s">
         <v>16</v>
       </c>
@@ -1517,7 +1517,7 @@
         <v>74.010000000000005</v>
       </c>
     </row>
-    <row r="13" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A13" s="5" t="s">
         <v>17</v>
       </c>
@@ -1579,7 +1579,7 @@
         <v>19.21</v>
       </c>
     </row>
-    <row r="14" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A14" s="5" t="s">
         <v>18</v>
       </c>
@@ -1641,7 +1641,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A15" s="5" t="s">
         <v>19</v>
       </c>
@@ -1703,7 +1703,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A16" s="5" t="s">
         <v>20</v>
       </c>
@@ -1765,7 +1765,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A17" s="5" t="s">
         <v>21</v>
       </c>
@@ -1827,7 +1827,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A18" s="8" t="s">
         <v>22</v>
       </c>
@@ -1889,7 +1889,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A19" s="5" t="s">
         <v>23</v>
       </c>
@@ -1951,7 +1951,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A20" s="5" t="s">
         <v>24</v>
       </c>
@@ -2021,9 +2021,9 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:C20"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -2034,7 +2034,7 @@
         <v>20.000000000000011</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" s="11" t="s">
         <v>3</v>
       </c>
@@ -2042,7 +2042,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" s="11" t="s">
         <v>5</v>
       </c>
@@ -2050,7 +2050,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" s="11" t="s">
         <v>6</v>
       </c>
@@ -2058,7 +2058,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" s="11" t="s">
         <v>7</v>
       </c>
@@ -2069,7 +2069,7 @@
         <v>11825.709472255599</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" s="11" t="s">
         <v>9</v>
       </c>
@@ -2080,7 +2080,7 @@
         <v>4024.640837013967</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" s="11" t="s">
         <v>10</v>
       </c>
@@ -2091,7 +2091,7 @@
         <v>894.50556158166398</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" s="11" t="s">
         <v>11</v>
       </c>
@@ -2102,7 +2102,7 @@
         <v>6906.5630736599669</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" s="5" t="s">
         <v>12</v>
       </c>
@@ -2113,7 +2113,7 @@
         <v>4.03</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" s="5" t="s">
         <v>14</v>
       </c>
@@ -2124,7 +2124,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" s="5" t="s">
         <v>15</v>
       </c>
@@ -2135,7 +2135,7 @@
         <v>1.78</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" s="5" t="s">
         <v>16</v>
       </c>
@@ -2146,7 +2146,7 @@
         <v>74.19</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" s="5" t="s">
         <v>17</v>
       </c>
@@ -2157,7 +2157,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" s="5" t="s">
         <v>18</v>
       </c>
@@ -2168,7 +2168,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15" s="5" t="s">
         <v>19</v>
       </c>
@@ -2179,7 +2179,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16" s="5" t="s">
         <v>20</v>
       </c>
@@ -2190,7 +2190,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" s="5" t="s">
         <v>21</v>
       </c>
@@ -2201,7 +2201,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" s="8" t="s">
         <v>22</v>
       </c>
@@ -2212,12 +2212,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" s="5" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20" s="5" t="s">
         <v>24</v>
       </c>
@@ -2230,12 +2230,12 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:P21"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="5" max="6" width="11" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -2285,22 +2285,22 @@
         <v>39.000000000000007</v>
       </c>
     </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A2" s="11" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A3" s="11" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A4" s="11" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A5" s="11" t="s">
         <v>7</v>
       </c>
@@ -2350,7 +2350,7 @@
         <v>5966.2428031122136</v>
       </c>
     </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A6" s="11" t="s">
         <v>9</v>
       </c>
@@ -2400,7 +2400,7 @@
         <v>2140.7099875659551</v>
       </c>
     </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A7" s="11" t="s">
         <v>10</v>
       </c>
@@ -2450,7 +2450,7 @@
         <v>451.27554153716352</v>
       </c>
     </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A8" s="11" t="s">
         <v>11</v>
       </c>
@@ -2500,7 +2500,7 @@
         <v>3374.2572740090959</v>
       </c>
     </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A9" s="5" t="s">
         <v>12</v>
       </c>
@@ -2550,7 +2550,7 @@
         <v>7.2</v>
       </c>
     </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A10" s="5" t="s">
         <v>14</v>
       </c>
@@ -2600,7 +2600,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A11" s="5" t="s">
         <v>15</v>
       </c>
@@ -2650,7 +2650,7 @@
         <v>3.47</v>
       </c>
     </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A12" s="5" t="s">
         <v>16</v>
       </c>
@@ -2700,7 +2700,7 @@
         <v>26.6</v>
       </c>
     </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A13" s="5" t="s">
         <v>17</v>
       </c>
@@ -2750,7 +2750,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A14" s="5" t="s">
         <v>18</v>
       </c>
@@ -2800,7 +2800,7 @@
         <v>42.73</v>
       </c>
     </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A15" s="5" t="s">
         <v>19</v>
       </c>
@@ -2850,7 +2850,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A16" s="5" t="s">
         <v>20</v>
       </c>
@@ -2900,7 +2900,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A17" s="5" t="s">
         <v>21</v>
       </c>
@@ -2950,7 +2950,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A18" s="8" t="s">
         <v>22</v>
       </c>
@@ -3000,17 +3000,17 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A19" s="5" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="20" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A20" s="5" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="21" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:16" x14ac:dyDescent="0.3">
       <c r="B21">
         <f t="shared" ref="B21:P21" si="0">B7/(B7+B6)</f>
         <v>0.18287975893375388</v>
@@ -3080,17 +3080,17 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:AG27"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="19.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.109375" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="10" bestFit="1" customWidth="1"/>
-    <col min="18" max="26" width="9.7109375" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="10.7109375" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="14.5703125" bestFit="1" customWidth="1"/>
-    <col min="29" max="32" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="18" max="26" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="14.5546875" bestFit="1" customWidth="1"/>
+    <col min="29" max="32" width="9.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -3191,7 +3191,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="2" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A2" s="11" t="s">
         <v>3</v>
       </c>
@@ -3292,7 +3292,7 @@
         <v>4.6570550596305296</v>
       </c>
     </row>
-    <row r="3" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A3" s="11" t="s">
         <v>5</v>
       </c>
@@ -3393,7 +3393,7 @@
         <v>1.804729825901729</v>
       </c>
     </row>
-    <row r="4" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A4" s="11" t="s">
         <v>6</v>
       </c>
@@ -3494,7 +3494,7 @@
         <v>0.44833772657454352</v>
       </c>
     </row>
-    <row r="5" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A5" s="11" t="s">
         <v>7</v>
       </c>
@@ -3595,7 +3595,7 @@
         <v>4473.5921132200983</v>
       </c>
     </row>
-    <row r="6" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A6" s="11" t="s">
         <v>9</v>
       </c>
@@ -3696,7 +3696,7 @@
         <v>1863.867735087701</v>
       </c>
     </row>
-    <row r="7" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A7" s="11" t="s">
         <v>10</v>
       </c>
@@ -3797,7 +3797,7 @@
         <v>350.2837743110498</v>
       </c>
     </row>
-    <row r="8" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A8" s="11" t="s">
         <v>11</v>
       </c>
@@ -3898,7 +3898,7 @@
         <v>2259.4406038213478</v>
       </c>
     </row>
-    <row r="9" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A9" s="5" t="s">
         <v>12</v>
       </c>
@@ -3999,7 +3999,7 @@
         <v>5.98</v>
       </c>
     </row>
-    <row r="10" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A10" s="5" t="s">
         <v>14</v>
       </c>
@@ -4100,7 +4100,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A11" s="5" t="s">
         <v>15</v>
       </c>
@@ -4201,7 +4201,7 @@
         <v>4.4400000000000004</v>
       </c>
     </row>
-    <row r="12" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A12" s="5" t="s">
         <v>16</v>
       </c>
@@ -4302,7 +4302,7 @@
         <v>32.64</v>
       </c>
     </row>
-    <row r="13" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A13" s="5" t="s">
         <v>17</v>
       </c>
@@ -4403,7 +4403,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="14" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A14" s="5" t="s">
         <v>18</v>
       </c>
@@ -4504,7 +4504,7 @@
         <v>36.94</v>
       </c>
     </row>
-    <row r="15" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A15" s="5" t="s">
         <v>19</v>
       </c>
@@ -4605,7 +4605,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A16" s="5" t="s">
         <v>20</v>
       </c>
@@ -4706,7 +4706,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A17" s="5" t="s">
         <v>21</v>
       </c>
@@ -4807,7 +4807,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A18" s="8" t="s">
         <v>22</v>
       </c>
@@ -4908,7 +4908,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A19" s="5" t="s">
         <v>23</v>
       </c>
@@ -5009,7 +5009,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A20" s="5" t="s">
         <v>24</v>
       </c>
@@ -5110,7 +5110,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:33" x14ac:dyDescent="0.3">
       <c r="B21">
         <f>($B$8-B8)/$B$8</f>
         <v>0</v>
@@ -5144,7 +5144,7 @@
         <v>0.4451696744770795</v>
       </c>
     </row>
-    <row r="22" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A22" s="5" t="s">
         <v>25</v>
       </c>
@@ -5213,7 +5213,7 @@
         <v>130.64444444444445</v>
       </c>
     </row>
-    <row r="23" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A23" s="5" t="s">
         <v>26</v>
       </c>
@@ -5282,7 +5282,7 @@
         <v>32.857538066085269</v>
       </c>
     </row>
-    <row r="24" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A24" s="5" t="s">
         <v>27</v>
       </c>
@@ -5351,7 +5351,7 @@
         <v>16.464264734829207</v>
       </c>
     </row>
-    <row r="25" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A25" s="5" t="s">
         <v>28</v>
       </c>
@@ -5420,9 +5420,9 @@
         <v>2.9878659712359878</v>
       </c>
     </row>
-    <row r="27" spans="1:33" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A27" s="5" t="s">
-        <v>29</v>
+        <v>37</v>
       </c>
       <c r="B27">
         <v>0.95</v>
@@ -5529,13 +5529,13 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:AD41"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="3" max="3" width="12.7109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -5597,31 +5597,31 @@
         <v>24</v>
       </c>
       <c r="W1" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="X1" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="X1" s="5" t="s">
+      <c r="Y1" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="Y1" s="5" t="s">
+      <c r="Z1" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="Z1" s="5" t="s">
+      <c r="AA1" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="AA1" s="5" t="s">
+      <c r="AB1" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="AB1" s="5" t="s">
+      <c r="AC1" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="AC1" s="5" t="s">
+      <c r="AD1" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="AD1" s="5" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="2" spans="1:30" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>50</v>
       </c>
@@ -5723,7 +5723,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>49.999999999999993</v>
       </c>
@@ -5825,7 +5825,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>50</v>
       </c>
@@ -5927,7 +5927,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>20</v>
       </c>
@@ -6029,7 +6029,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>20</v>
       </c>
@@ -6131,7 +6131,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>20</v>
       </c>
@@ -6233,7 +6233,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>20</v>
       </c>
@@ -6335,7 +6335,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>23</v>
       </c>
@@ -6437,7 +6437,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>25</v>
       </c>
@@ -6539,7 +6539,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>28</v>
       </c>
@@ -6641,7 +6641,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>30</v>
       </c>
@@ -6743,7 +6743,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>33</v>
       </c>
@@ -6845,7 +6845,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>35.000000000000007</v>
       </c>
@@ -6947,7 +6947,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>40</v>
       </c>
@@ -7049,7 +7049,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>45</v>
       </c>
@@ -7151,7 +7151,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>50</v>
       </c>
@@ -7253,7 +7253,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A18" s="5"/>
       <c r="E18" s="16"/>
       <c r="I18" s="17"/>
@@ -7268,7 +7268,7 @@
       <c r="R18" s="17"/>
       <c r="U18" s="16"/>
     </row>
-    <row r="19" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A19" s="5"/>
       <c r="I19" s="18"/>
       <c r="K19" s="18"/>
@@ -7279,7 +7279,7 @@
       <c r="Q19" s="18"/>
       <c r="R19" s="18"/>
     </row>
-    <row r="20" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:30" x14ac:dyDescent="0.3">
       <c r="C20" s="23"/>
       <c r="I20" s="16"/>
       <c r="J20" s="16"/>
@@ -7292,7 +7292,7 @@
       <c r="Q20" s="16"/>
       <c r="R20" s="16"/>
     </row>
-    <row r="21" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:30" x14ac:dyDescent="0.3">
       <c r="C21" s="23"/>
       <c r="I21" s="16"/>
       <c r="J21" s="16"/>
@@ -7305,7 +7305,7 @@
       <c r="Q21" s="16"/>
       <c r="R21" s="16"/>
     </row>
-    <row r="22" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:30" x14ac:dyDescent="0.3">
       <c r="I22" s="16"/>
       <c r="J22" s="16"/>
       <c r="K22" s="16"/>
@@ -7317,15 +7317,15 @@
       <c r="Q22" s="16"/>
       <c r="R22" s="16"/>
     </row>
-    <row r="23" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:30" x14ac:dyDescent="0.3">
       <c r="L23" s="16"/>
       <c r="M23" s="16"/>
     </row>
-    <row r="24" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:30" x14ac:dyDescent="0.3">
       <c r="L24" s="21"/>
       <c r="M24" s="21"/>
     </row>
-    <row r="25" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:30" x14ac:dyDescent="0.3">
       <c r="I25" s="19"/>
       <c r="J25" s="19"/>
       <c r="K25" s="19"/>
@@ -7343,7 +7343,7 @@
       <c r="W25" s="14"/>
       <c r="X25" s="14"/>
     </row>
-    <row r="26" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:30" x14ac:dyDescent="0.3">
       <c r="I26" s="20"/>
       <c r="J26" s="18"/>
       <c r="K26" s="18"/>
@@ -7361,7 +7361,7 @@
       <c r="W26" s="14"/>
       <c r="X26" s="14"/>
     </row>
-    <row r="27" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:30" x14ac:dyDescent="0.3">
       <c r="I27" s="18"/>
       <c r="J27" s="18"/>
       <c r="K27" s="18"/>
@@ -7379,7 +7379,7 @@
       <c r="W27" s="14"/>
       <c r="X27" s="14"/>
     </row>
-    <row r="28" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:30" x14ac:dyDescent="0.3">
       <c r="I28" s="18"/>
       <c r="J28" s="20"/>
       <c r="K28" s="18"/>
@@ -7397,7 +7397,7 @@
       <c r="W28" s="15"/>
       <c r="X28" s="15"/>
     </row>
-    <row r="29" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:30" x14ac:dyDescent="0.3">
       <c r="I29" s="18"/>
       <c r="J29" s="18"/>
       <c r="K29" s="18"/>
@@ -7415,7 +7415,7 @@
       <c r="W29" s="15"/>
       <c r="X29" s="15"/>
     </row>
-    <row r="30" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:30" x14ac:dyDescent="0.3">
       <c r="I30" s="20"/>
       <c r="J30" s="18"/>
       <c r="K30" s="18"/>
@@ -7433,7 +7433,7 @@
       <c r="W30" s="15"/>
       <c r="X30" s="15"/>
     </row>
-    <row r="31" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:30" x14ac:dyDescent="0.3">
       <c r="S31" s="15"/>
       <c r="T31" s="15"/>
       <c r="U31" s="15"/>
@@ -7441,7 +7441,7 @@
       <c r="W31" s="15"/>
       <c r="X31" s="15"/>
     </row>
-    <row r="32" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:30" x14ac:dyDescent="0.3">
       <c r="J32" s="14"/>
       <c r="K32" s="14"/>
       <c r="L32" s="14"/>
@@ -7458,7 +7458,7 @@
       <c r="W32" s="14"/>
       <c r="X32" s="14"/>
     </row>
-    <row r="33" spans="10:24" x14ac:dyDescent="0.25">
+    <row r="33" spans="10:24" x14ac:dyDescent="0.3">
       <c r="J33" s="14"/>
       <c r="K33" s="14"/>
       <c r="L33" s="14"/>
@@ -7475,7 +7475,7 @@
       <c r="W33" s="14"/>
       <c r="X33" s="14"/>
     </row>
-    <row r="34" spans="10:24" x14ac:dyDescent="0.25">
+    <row r="34" spans="10:24" x14ac:dyDescent="0.3">
       <c r="J34" s="14"/>
       <c r="K34" s="14"/>
       <c r="L34" s="14"/>
@@ -7492,7 +7492,7 @@
       <c r="W34" s="14"/>
       <c r="X34" s="14"/>
     </row>
-    <row r="35" spans="10:24" x14ac:dyDescent="0.25">
+    <row r="35" spans="10:24" x14ac:dyDescent="0.3">
       <c r="J35" s="14"/>
       <c r="K35" s="14"/>
       <c r="L35" s="14"/>
@@ -7509,7 +7509,7 @@
       <c r="W35" s="14"/>
       <c r="X35" s="14"/>
     </row>
-    <row r="36" spans="10:24" x14ac:dyDescent="0.25">
+    <row r="36" spans="10:24" x14ac:dyDescent="0.3">
       <c r="J36" s="14"/>
       <c r="K36" s="14"/>
       <c r="L36" s="14"/>
@@ -7526,7 +7526,7 @@
       <c r="W36" s="14"/>
       <c r="X36" s="14"/>
     </row>
-    <row r="37" spans="10:24" x14ac:dyDescent="0.25">
+    <row r="37" spans="10:24" x14ac:dyDescent="0.3">
       <c r="J37" s="14"/>
       <c r="K37" s="14"/>
       <c r="L37" s="14"/>
@@ -7543,7 +7543,7 @@
       <c r="W37" s="14"/>
       <c r="X37" s="14"/>
     </row>
-    <row r="38" spans="10:24" x14ac:dyDescent="0.25">
+    <row r="38" spans="10:24" x14ac:dyDescent="0.3">
       <c r="J38" s="14"/>
       <c r="K38" s="14"/>
       <c r="L38" s="14"/>
@@ -7560,7 +7560,7 @@
       <c r="W38" s="14"/>
       <c r="X38" s="14"/>
     </row>
-    <row r="39" spans="10:24" x14ac:dyDescent="0.25">
+    <row r="39" spans="10:24" x14ac:dyDescent="0.3">
       <c r="J39" s="14"/>
       <c r="K39" s="14"/>
       <c r="L39" s="14"/>
@@ -7577,7 +7577,7 @@
       <c r="W39" s="14"/>
       <c r="X39" s="14"/>
     </row>
-    <row r="40" spans="10:24" x14ac:dyDescent="0.25">
+    <row r="40" spans="10:24" x14ac:dyDescent="0.3">
       <c r="J40" s="14"/>
       <c r="K40" s="14"/>
       <c r="L40" s="14"/>
@@ -7594,7 +7594,7 @@
       <c r="W40" s="14"/>
       <c r="X40" s="14"/>
     </row>
-    <row r="41" spans="10:24" x14ac:dyDescent="0.25">
+    <row r="41" spans="10:24" x14ac:dyDescent="0.3">
       <c r="J41" s="14"/>
       <c r="K41" s="14"/>
       <c r="L41" s="14"/>
@@ -7619,16 +7619,16 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:AD33"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="5" max="6" width="11" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="10.6640625" bestFit="1" customWidth="1"/>
     <col min="23" max="23" width="12" bestFit="1" customWidth="1"/>
     <col min="24" max="24" width="10" bestFit="1" customWidth="1"/>
     <col min="28" max="28" width="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -7690,31 +7690,31 @@
         <v>24</v>
       </c>
       <c r="W1" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="X1" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="X1" s="5" t="s">
+      <c r="Y1" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="Y1" s="5" t="s">
+      <c r="Z1" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="Z1" s="5" t="s">
+      <c r="AA1" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="AA1" s="5" t="s">
+      <c r="AB1" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="AB1" s="5" t="s">
+      <c r="AC1" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="AC1" s="5" t="s">
+      <c r="AD1" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="AD1" s="5" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="2" spans="1:30" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>40</v>
       </c>
@@ -7801,7 +7801,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>30</v>
       </c>
@@ -7888,7 +7888,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>24.999999999999989</v>
       </c>
@@ -7975,7 +7975,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>20</v>
       </c>
@@ -8062,7 +8062,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>19</v>
       </c>
@@ -8149,7 +8149,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>49.999999999999993</v>
       </c>
@@ -8236,7 +8236,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>45</v>
       </c>
@@ -8323,7 +8323,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>33</v>
       </c>
@@ -8410,7 +8410,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>28</v>
       </c>
@@ -8497,7 +8497,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>23</v>
       </c>
@@ -8584,7 +8584,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>35</v>
       </c>
@@ -8671,7 +8671,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>36</v>
       </c>
@@ -8758,7 +8758,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>37.000000000000007</v>
       </c>
@@ -8845,7 +8845,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>38</v>
       </c>
@@ -8932,7 +8932,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>39.000000000000007</v>
       </c>
@@ -9019,12 +9019,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A17" s="5"/>
       <c r="E17" s="16"/>
       <c r="V17" s="16"/>
     </row>
-    <row r="18" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:22" x14ac:dyDescent="0.3">
       <c r="I18" s="17"/>
       <c r="J18" s="17"/>
       <c r="K18" s="17"/>
@@ -9036,7 +9036,7 @@
       <c r="Q18" s="17"/>
       <c r="R18" s="17"/>
     </row>
-    <row r="19" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:22" x14ac:dyDescent="0.3">
       <c r="I19" s="18"/>
       <c r="K19" s="18"/>
       <c r="L19" s="21"/>
@@ -9046,7 +9046,7 @@
       <c r="Q19" s="18"/>
       <c r="R19" s="18"/>
     </row>
-    <row r="20" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:22" x14ac:dyDescent="0.3">
       <c r="I20" s="16"/>
       <c r="J20" s="16"/>
       <c r="K20" s="16"/>
@@ -9058,7 +9058,7 @@
       <c r="Q20" s="16"/>
       <c r="R20" s="16"/>
     </row>
-    <row r="21" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:22" x14ac:dyDescent="0.3">
       <c r="I21" s="16"/>
       <c r="J21" s="16"/>
       <c r="K21" s="16"/>
@@ -9070,7 +9070,7 @@
       <c r="Q21" s="16"/>
       <c r="R21" s="16"/>
     </row>
-    <row r="22" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:22" x14ac:dyDescent="0.3">
       <c r="I22" s="16"/>
       <c r="J22" s="16"/>
       <c r="K22" s="16"/>
@@ -9082,15 +9082,15 @@
       <c r="Q22" s="16"/>
       <c r="R22" s="16"/>
     </row>
-    <row r="23" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:22" x14ac:dyDescent="0.3">
       <c r="L23" s="16"/>
       <c r="M23" s="16"/>
     </row>
-    <row r="24" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:22" x14ac:dyDescent="0.3">
       <c r="L24" s="21"/>
       <c r="M24" s="21"/>
     </row>
-    <row r="25" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:22" x14ac:dyDescent="0.3">
       <c r="I25" s="19"/>
       <c r="J25" s="19"/>
       <c r="K25" s="19"/>
@@ -9102,7 +9102,7 @@
       <c r="Q25" s="19"/>
       <c r="R25" s="19"/>
     </row>
-    <row r="26" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:22" x14ac:dyDescent="0.3">
       <c r="I26" s="20"/>
       <c r="J26" s="18"/>
       <c r="K26" s="18"/>
@@ -9114,7 +9114,7 @@
       <c r="Q26" s="18"/>
       <c r="R26" s="18"/>
     </row>
-    <row r="27" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:22" x14ac:dyDescent="0.3">
       <c r="I27" s="18"/>
       <c r="J27" s="18"/>
       <c r="K27" s="18"/>
@@ -9126,7 +9126,7 @@
       <c r="Q27" s="18"/>
       <c r="R27" s="18"/>
     </row>
-    <row r="28" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:22" x14ac:dyDescent="0.3">
       <c r="I28" s="18"/>
       <c r="J28" s="20"/>
       <c r="K28" s="18"/>
@@ -9138,7 +9138,7 @@
       <c r="Q28" s="18"/>
       <c r="R28" s="18"/>
     </row>
-    <row r="29" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:22" x14ac:dyDescent="0.3">
       <c r="I29" s="18"/>
       <c r="J29" s="18"/>
       <c r="K29" s="18"/>
@@ -9150,7 +9150,7 @@
       <c r="Q29" s="18"/>
       <c r="R29" s="18"/>
     </row>
-    <row r="30" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:22" x14ac:dyDescent="0.3">
       <c r="I30" s="20"/>
       <c r="J30" s="18"/>
       <c r="K30" s="18"/>
@@ -9162,7 +9162,7 @@
       <c r="Q30" s="20"/>
       <c r="R30" s="20"/>
     </row>
-    <row r="33" spans="5:5" x14ac:dyDescent="0.25">
+    <row r="33" spans="5:5" x14ac:dyDescent="0.3">
       <c r="E33" s="16"/>
     </row>
   </sheetData>
@@ -9173,9 +9173,9 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:Y50"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -9237,10 +9237,10 @@
         <v>24</v>
       </c>
       <c r="U1" s="5" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="2" spans="1:25" x14ac:dyDescent="0.25">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="2" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>20.000000000000011</v>
       </c>
@@ -9305,7 +9305,7 @@
         <v>0.99</v>
       </c>
     </row>
-    <row r="3" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>20</v>
       </c>
@@ -9374,7 +9374,7 @@
       <c r="X3" s="15"/>
       <c r="Y3" s="15"/>
     </row>
-    <row r="4" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>20</v>
       </c>
@@ -9439,7 +9439,7 @@
         <v>0.9</v>
       </c>
     </row>
-    <row r="5" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>20.000000000000011</v>
       </c>
@@ -9504,7 +9504,7 @@
         <v>0.8</v>
       </c>
     </row>
-    <row r="6" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>20.000000000000011</v>
       </c>
@@ -9569,7 +9569,7 @@
         <v>0.7</v>
       </c>
     </row>
-    <row r="7" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>20.000000000000011</v>
       </c>
@@ -9634,7 +9634,7 @@
         <v>0.6</v>
       </c>
     </row>
-    <row r="8" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>20</v>
       </c>
@@ -9699,7 +9699,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="9" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>20</v>
       </c>
@@ -9764,7 +9764,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="10" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>20.000000000000011</v>
       </c>
@@ -9829,7 +9829,7 @@
         <v>0.3</v>
       </c>
     </row>
-    <row r="11" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>20</v>
       </c>
@@ -9894,7 +9894,7 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="12" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>20</v>
       </c>
@@ -9959,7 +9959,7 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="13" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>20.000000000000011</v>
       </c>
@@ -10024,7 +10024,7 @@
         <v>0.05</v>
       </c>
     </row>
-    <row r="14" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>20</v>
       </c>
@@ -10089,7 +10089,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="15" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>50</v>
       </c>
@@ -10154,7 +10154,7 @@
         <v>0.99</v>
       </c>
     </row>
-    <row r="16" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>50</v>
       </c>
@@ -10219,7 +10219,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="17" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>50</v>
       </c>
@@ -10284,7 +10284,7 @@
         <v>0.05</v>
       </c>
     </row>
-    <row r="18" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>50</v>
       </c>
@@ -10349,7 +10349,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="19" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A19" s="14"/>
       <c r="B19" s="14"/>
       <c r="C19" s="14"/>
@@ -10369,7 +10369,7 @@
       <c r="Q19" s="12"/>
       <c r="R19" s="12"/>
     </row>
-    <row r="20" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A20" s="14"/>
       <c r="B20" s="14"/>
       <c r="C20" s="14"/>
@@ -10389,7 +10389,7 @@
       <c r="Q20" s="12"/>
       <c r="R20" s="12"/>
     </row>
-    <row r="21" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A21" s="14"/>
       <c r="C21" s="14"/>
       <c r="D21" s="14"/>
@@ -10409,7 +10409,7 @@
       <c r="R21" s="12"/>
       <c r="S21" s="12"/>
     </row>
-    <row r="22" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:21" x14ac:dyDescent="0.3">
       <c r="C22" s="14"/>
       <c r="D22" s="14"/>
       <c r="E22" s="14"/>
@@ -10428,7 +10428,7 @@
       <c r="R22" s="12"/>
       <c r="S22" s="12"/>
     </row>
-    <row r="23" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:21" x14ac:dyDescent="0.3">
       <c r="C23" s="14"/>
       <c r="D23" s="14"/>
       <c r="E23" s="14"/>
@@ -10447,7 +10447,7 @@
       <c r="R23" s="12"/>
       <c r="S23" s="12"/>
     </row>
-    <row r="24" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:21" x14ac:dyDescent="0.3">
       <c r="C24" s="14"/>
       <c r="D24" s="14"/>
       <c r="E24" s="14"/>
@@ -10466,7 +10466,7 @@
       <c r="R24" s="12"/>
       <c r="S24" s="12"/>
     </row>
-    <row r="25" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:21" x14ac:dyDescent="0.3">
       <c r="C25" s="14"/>
       <c r="D25" s="14"/>
       <c r="E25" s="14"/>
@@ -10485,7 +10485,7 @@
       <c r="R25" s="12"/>
       <c r="S25" s="12"/>
     </row>
-    <row r="26" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:21" x14ac:dyDescent="0.3">
       <c r="C26" s="14"/>
       <c r="D26" s="14"/>
       <c r="E26" s="14"/>
@@ -10504,7 +10504,7 @@
       <c r="R26" s="12"/>
       <c r="S26" s="12"/>
     </row>
-    <row r="27" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:21" x14ac:dyDescent="0.3">
       <c r="C27" s="14"/>
       <c r="D27" s="14"/>
       <c r="E27" s="14"/>
@@ -10523,7 +10523,7 @@
       <c r="R27" s="12"/>
       <c r="S27" s="12"/>
     </row>
-    <row r="28" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:21" x14ac:dyDescent="0.3">
       <c r="C28" s="14"/>
       <c r="D28" s="14"/>
       <c r="E28" s="14"/>
@@ -10542,7 +10542,7 @@
       <c r="R28" s="12"/>
       <c r="S28" s="12"/>
     </row>
-    <row r="29" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:21" x14ac:dyDescent="0.3">
       <c r="C29" s="14"/>
       <c r="D29" s="14"/>
       <c r="E29" s="14"/>
@@ -10561,7 +10561,7 @@
       <c r="R29" s="12"/>
       <c r="S29" s="12"/>
     </row>
-    <row r="30" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:21" x14ac:dyDescent="0.3">
       <c r="C30" s="14"/>
       <c r="D30" s="14"/>
       <c r="E30" s="14"/>
@@ -10580,7 +10580,7 @@
       <c r="R30" s="12"/>
       <c r="S30" s="12"/>
     </row>
-    <row r="31" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:21" x14ac:dyDescent="0.3">
       <c r="C31" s="14"/>
       <c r="D31" s="14"/>
       <c r="E31" s="14"/>
@@ -10599,7 +10599,7 @@
       <c r="R31" s="12"/>
       <c r="S31" s="12"/>
     </row>
-    <row r="32" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:21" x14ac:dyDescent="0.3">
       <c r="C32" s="14"/>
       <c r="D32" s="14"/>
       <c r="E32" s="14"/>
@@ -10618,7 +10618,7 @@
       <c r="R32" s="12"/>
       <c r="S32" s="12"/>
     </row>
-    <row r="33" spans="3:23" x14ac:dyDescent="0.25">
+    <row r="33" spans="3:23" x14ac:dyDescent="0.3">
       <c r="C33" s="14"/>
       <c r="D33" s="14"/>
       <c r="E33" s="14"/>
@@ -10637,7 +10637,7 @@
       <c r="R33" s="12"/>
       <c r="S33" s="12"/>
     </row>
-    <row r="34" spans="3:23" x14ac:dyDescent="0.25">
+    <row r="34" spans="3:23" x14ac:dyDescent="0.3">
       <c r="C34" s="14"/>
       <c r="D34" s="14"/>
       <c r="E34" s="14"/>
@@ -10656,7 +10656,7 @@
       <c r="R34" s="12"/>
       <c r="S34" s="12"/>
     </row>
-    <row r="35" spans="3:23" x14ac:dyDescent="0.25">
+    <row r="35" spans="3:23" x14ac:dyDescent="0.3">
       <c r="C35" s="14"/>
       <c r="D35" s="14"/>
       <c r="E35" s="14"/>
@@ -10675,7 +10675,7 @@
       <c r="R35" s="12"/>
       <c r="S35" s="12"/>
     </row>
-    <row r="36" spans="3:23" x14ac:dyDescent="0.25">
+    <row r="36" spans="3:23" x14ac:dyDescent="0.3">
       <c r="C36" s="14"/>
       <c r="D36" s="14"/>
       <c r="E36" s="14"/>
@@ -10694,7 +10694,7 @@
       <c r="R36" s="12"/>
       <c r="S36" s="12"/>
     </row>
-    <row r="37" spans="3:23" x14ac:dyDescent="0.25">
+    <row r="37" spans="3:23" x14ac:dyDescent="0.3">
       <c r="C37" s="14"/>
       <c r="D37" s="14"/>
       <c r="E37" s="14"/>
@@ -10713,7 +10713,7 @@
       <c r="R37" s="12"/>
       <c r="S37" s="12"/>
     </row>
-    <row r="38" spans="3:23" x14ac:dyDescent="0.25">
+    <row r="38" spans="3:23" x14ac:dyDescent="0.3">
       <c r="C38" s="14"/>
       <c r="D38" s="14"/>
       <c r="E38" s="14"/>
@@ -10732,7 +10732,7 @@
       <c r="R38" s="12"/>
       <c r="S38" s="12"/>
     </row>
-    <row r="39" spans="3:23" x14ac:dyDescent="0.25">
+    <row r="39" spans="3:23" x14ac:dyDescent="0.3">
       <c r="C39" s="14"/>
       <c r="D39" s="14"/>
       <c r="E39" s="14"/>
@@ -10751,7 +10751,7 @@
       <c r="R39" s="12"/>
       <c r="S39" s="12"/>
     </row>
-    <row r="40" spans="3:23" x14ac:dyDescent="0.25">
+    <row r="40" spans="3:23" x14ac:dyDescent="0.3">
       <c r="C40" s="14"/>
       <c r="D40" s="14"/>
       <c r="E40" s="14"/>
@@ -10770,7 +10770,7 @@
       <c r="R40" s="12"/>
       <c r="S40" s="12"/>
     </row>
-    <row r="41" spans="3:23" x14ac:dyDescent="0.25">
+    <row r="41" spans="3:23" x14ac:dyDescent="0.3">
       <c r="C41" s="14"/>
       <c r="D41" s="14"/>
       <c r="E41" s="14"/>
@@ -10789,7 +10789,7 @@
       <c r="R41" s="12"/>
       <c r="S41" s="12"/>
     </row>
-    <row r="42" spans="3:23" x14ac:dyDescent="0.25">
+    <row r="42" spans="3:23" x14ac:dyDescent="0.3">
       <c r="C42" s="14"/>
       <c r="D42" s="14"/>
       <c r="E42" s="14"/>
@@ -10808,7 +10808,7 @@
       <c r="R42" s="12"/>
       <c r="S42" s="12"/>
     </row>
-    <row r="43" spans="3:23" x14ac:dyDescent="0.25">
+    <row r="43" spans="3:23" x14ac:dyDescent="0.3">
       <c r="C43" s="14"/>
       <c r="D43" s="14"/>
       <c r="E43" s="14"/>
@@ -10827,7 +10827,7 @@
       <c r="R43" s="12"/>
       <c r="S43" s="12"/>
     </row>
-    <row r="44" spans="3:23" x14ac:dyDescent="0.25">
+    <row r="44" spans="3:23" x14ac:dyDescent="0.3">
       <c r="C44" s="14"/>
       <c r="D44" s="14"/>
       <c r="E44" s="14"/>
@@ -10846,7 +10846,7 @@
       <c r="R44" s="12"/>
       <c r="S44" s="12"/>
     </row>
-    <row r="45" spans="3:23" x14ac:dyDescent="0.25">
+    <row r="45" spans="3:23" x14ac:dyDescent="0.3">
       <c r="C45" s="14"/>
       <c r="D45" s="14"/>
       <c r="E45" s="14"/>
@@ -10865,7 +10865,7 @@
       <c r="R45" s="12"/>
       <c r="S45" s="12"/>
     </row>
-    <row r="46" spans="3:23" x14ac:dyDescent="0.25">
+    <row r="46" spans="3:23" x14ac:dyDescent="0.3">
       <c r="C46" s="14"/>
       <c r="D46" s="14"/>
       <c r="E46" s="14"/>
@@ -10884,7 +10884,7 @@
       <c r="R46" s="12"/>
       <c r="S46" s="12"/>
     </row>
-    <row r="47" spans="3:23" x14ac:dyDescent="0.25">
+    <row r="47" spans="3:23" x14ac:dyDescent="0.3">
       <c r="C47" s="14"/>
       <c r="D47" s="14"/>
       <c r="E47" s="14"/>
@@ -10903,7 +10903,7 @@
       <c r="R47" s="12"/>
       <c r="S47" s="12"/>
     </row>
-    <row r="48" spans="3:23" x14ac:dyDescent="0.25">
+    <row r="48" spans="3:23" x14ac:dyDescent="0.3">
       <c r="E48" s="14"/>
       <c r="F48" s="14"/>
       <c r="G48" s="14"/>
@@ -10924,7 +10924,7 @@
       <c r="V48" s="14"/>
       <c r="W48" s="14"/>
     </row>
-    <row r="49" spans="5:23" x14ac:dyDescent="0.25">
+    <row r="49" spans="5:23" x14ac:dyDescent="0.3">
       <c r="E49" s="14"/>
       <c r="F49" s="14"/>
       <c r="G49" s="14"/>
@@ -10945,7 +10945,7 @@
       <c r="V49" s="14"/>
       <c r="W49" s="14"/>
     </row>
-    <row r="50" spans="5:23" x14ac:dyDescent="0.25">
+    <row r="50" spans="5:23" x14ac:dyDescent="0.3">
       <c r="E50" s="14"/>
       <c r="F50" s="14"/>
       <c r="G50" s="14"/>

</xml_diff>